<commit_message>
Rebuild existing working files from the same generator as the new maps.
Keeps the spreadsheet blanks in lockstep with scripts/build-working-files.py after the CRM and vendor sheets were added.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/gtm-sales-capacity.xlsx
+++ b/templates/gtm-sales-capacity.xlsx
@@ -815,7 +815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -831,7 +831,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>List people. Ramp months with start date after month 1 carry zero quota until ramped.</t>
+          <t>List people. Start month and ramp are inputs. Payroll ≠ quota-bearing.</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1022,7 @@
   </sheetData>
   <autoFilter ref="A3:H3"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>